<commit_message>
Address code review feedback: fix imports, make path configurable, use DRY principle for dropdown options
Co-authored-by: staengel <58119858+staengel@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/Kundenüberwachung_Vorlage.xlsx
+++ b/Kundenüberwachung_Vorlage.xlsx
@@ -668,40 +668,40 @@
     <dataValidation sqref="D2:D1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Ungültige Eingabe" error="Bitte wählen Sie eine Kategorie aus der Liste" type="list">
       <formula1>=Kategorien!$A$2:$A$7</formula1>
     </dataValidation>
-    <dataValidation sqref="E2" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Ungültige Eingabe" error="Bitte wählen Sie einen Wert aus der Liste" type="list">
+    <dataValidation sqref="E2" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Ungültige Eingabe" error="Bitte wählen Sie einen Wert für Overlap aus der Liste" type="list">
       <formula1>"60/60,80/80,70/70"</formula1>
     </dataValidation>
-    <dataValidation sqref="F2" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Ungültige Eingabe" error="Bitte wählen Sie einen Wert aus der Liste" type="list">
+    <dataValidation sqref="F2" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Ungültige Eingabe" error="Bitte wählen Sie einen Wert für Kamera aus der Liste" type="list">
       <formula1>"RGB,Multispektral,Thermal"</formula1>
     </dataValidation>
-    <dataValidation sqref="G2" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Ungültige Eingabe" error="Bitte wählen Sie einen Wert aus der Liste" type="list">
+    <dataValidation sqref="G2" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Ungültige Eingabe" error="Bitte wählen Sie einen Wert für Auflösung aus der Liste" type="list">
       <formula1>"20MP,45MP,100MP"</formula1>
     </dataValidation>
-    <dataValidation sqref="H2" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Ungültige Eingabe" error="Bitte wählen Sie einen Wert aus der Liste" type="list">
+    <dataValidation sqref="H2" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Ungültige Eingabe" error="Bitte wählen Sie einen Wert für Flughöhe aus der Liste" type="list">
       <formula1>"50m,100m,120m,150m"</formula1>
     </dataValidation>
-    <dataValidation sqref="E3" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="E3" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Ungültige Eingabe" error="Bitte wählen Sie einen Wert für Anzahl Drohnen aus der Liste" type="list">
       <formula1>"10,25,50,100,200"</formula1>
     </dataValidation>
-    <dataValidation sqref="F3" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="F3" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Ungültige Eingabe" error="Bitte wählen Sie einen Wert für Dauer (Min) aus der Liste" type="list">
       <formula1>"5,10,15,20,30"</formula1>
     </dataValidation>
-    <dataValidation sqref="G3" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="G3" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Ungültige Eingabe" error="Bitte wählen Sie einen Wert für Musik aus der Liste" type="list">
       <formula1>"Ja,Nein"</formula1>
     </dataValidation>
-    <dataValidation sqref="H3" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="H3" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Ungültige Eingabe" error="Bitte wählen Sie einen Wert für Indoor/Outdoor aus der Liste" type="list">
       <formula1>"Indoor,Outdoor,Beides"</formula1>
     </dataValidation>
-    <dataValidation sqref="E4" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="E4" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Ungültige Eingabe" error="Bitte wählen Sie einen Wert für Detailgrad aus der Liste" type="list">
       <formula1>"Niedrig,Mittel,Hoch,Sehr Hoch"</formula1>
     </dataValidation>
-    <dataValidation sqref="F4" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="F4" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Ungültige Eingabe" error="Bitte wählen Sie einen Wert für Format aus der Liste" type="list">
       <formula1>"OBJ,FBX,STL,GLTF"</formula1>
     </dataValidation>
-    <dataValidation sqref="G4" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="G4" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Ungültige Eingabe" error="Bitte wählen Sie einen Wert für Texturierung aus der Liste" type="list">
       <formula1>"Ja,Nein"</formula1>
     </dataValidation>
-    <dataValidation sqref="H4" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="H4" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Ungültige Eingabe" error="Bitte wählen Sie einen Wert für Polygonanzahl aus der Liste" type="list">
       <formula1>"Low Poly,Medium Poly,High Poly"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>